<commit_message>
updates by claude to address baselvl vs. background issue; also small bug fix (2)
</commit_message>
<xml_diff>
--- a/Example_data/OUTPUT-1channel_frozen/data_leaf_damage_singlemetrics.xlsx
+++ b/Example_data/OUTPUT-1channel_frozen/data_leaf_damage_singlemetrics.xlsx
@@ -504,7 +504,7 @@
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>background_dmg</t>
+          <t>baselvl_dmg</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
         <v>78</v>
       </c>
       <c r="Q2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R2" t="n">
         <v>39</v>

</xml_diff>

<commit_message>
version 1.0 of improved analysis pipeline
</commit_message>
<xml_diff>
--- a/Example_data/OUTPUT-1channel_frozen/data_leaf_damage_singlemetrics.xlsx
+++ b/Example_data/OUTPUT-1channel_frozen/data_leaf_damage_singlemetrics.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S5"/>
+  <dimension ref="A1:AC5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,82 +434,132 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>damage_found</t>
+          <t>leaf_roundness</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>analysis_status</t>
+          <t>total_leaf_size_px</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>leaf_roundness</t>
+          <t>total_leaf_size_cm2</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>total_nearest_island_distances</t>
+          <t>threshold_val_leaf</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>mean_nearest_island_distance</t>
+          <t>background_leaf</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>island_counts</t>
+          <t>baselvl_dmg</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>total_leaf_size_px</t>
+          <t>mean_dmg_signal</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>total_leaf_size_cm2</t>
+          <t>damage_found_leafthr</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>total_damage_area_px</t>
+          <t>analysis_status_leafthr</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>total_damage_area_cm2</t>
+          <t>threshold_val_dmg_leafthr</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>total_damage_percentage</t>
+          <t>island_counts_leafthr</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>threshold_val_leaf</t>
+          <t>total_nearest_island_distances_leafthr</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>threshold_val_dmg</t>
+          <t>mean_nearest_island_distance_leafthr</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>background_leaf</t>
+          <t>total_damage_area_px_leafthr</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>baselvl_dmg</t>
+          <t>total_damage_area_cm2_leafthr</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>mean_dmg_signal</t>
+          <t>total_damage_percentage_leafthr</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>reference_condition</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>damage_found_refthr</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>analysis_status_refthr</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>threshold_val_dmg_refthr</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>island_counts_refthr</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>total_nearest_island_distances_refthr</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>mean_nearest_island_distance_refthr</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>total_damage_area_px_refthr</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>total_damage_area_cm2_refthr</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>total_damage_percentage_refthr</t>
         </is>
       </c>
     </row>
@@ -527,55 +577,89 @@
       <c r="C2" t="b">
         <v>1</v>
       </c>
-      <c r="D2" t="b">
-        <v>1</v>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="D2" t="n">
+        <v>0.8822018881922326</v>
+      </c>
+      <c r="E2" t="n">
+        <v>26847</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1.564419322883282</v>
+      </c>
+      <c r="G2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>39</v>
+      </c>
+      <c r="J2" t="n">
+        <v>58.71147614258577</v>
+      </c>
+      <c r="K2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>0.8822018881922326</v>
-      </c>
-      <c r="G2" t="n">
+      <c r="M2" t="n">
+        <v>78</v>
+      </c>
+      <c r="N2" t="n">
+        <v>26</v>
+      </c>
+      <c r="O2" t="n">
         <v>199.2340063194676</v>
       </c>
-      <c r="H2" t="n">
+      <c r="P2" t="n">
         <v>7.6628463969026</v>
       </c>
-      <c r="I2" t="n">
-        <v>26</v>
-      </c>
-      <c r="J2" t="n">
-        <v>26847</v>
-      </c>
-      <c r="K2" t="n">
-        <v>1.564419322883282</v>
-      </c>
-      <c r="L2" t="n">
+      <c r="Q2" t="n">
         <v>4731</v>
       </c>
-      <c r="M2" t="n">
+      <c r="R2" t="n">
         <v>0.2756832352427015</v>
       </c>
-      <c r="N2" t="n">
+      <c r="S2" t="n">
         <v>17.62208067940552</v>
       </c>
-      <c r="O2" t="n">
-        <v>5</v>
-      </c>
-      <c r="P2" t="n">
-        <v>78</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>1</v>
-      </c>
-      <c r="R2" t="n">
-        <v>39</v>
-      </c>
-      <c r="S2" t="n">
-        <v>58.71147614258577</v>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Ctrl</t>
+        </is>
+      </c>
+      <c r="U2" t="b">
+        <v>1</v>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="W2" t="n">
+        <v>106</v>
+      </c>
+      <c r="X2" t="n">
+        <v>14</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>166.6347844206641</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>11.90248460147601</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>2657</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>0.1548278072373405</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>9.896822736246136</v>
       </c>
     </row>
     <row r="3">
@@ -592,55 +676,89 @@
       <c r="C3" t="b">
         <v>1</v>
       </c>
-      <c r="D3" t="b">
-        <v>1</v>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="D3" t="n">
+        <v>0.8547185984544441</v>
+      </c>
+      <c r="E3" t="n">
+        <v>23287</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.356972204416992</v>
+      </c>
+      <c r="G3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" t="n">
+        <v>67</v>
+      </c>
+      <c r="J3" t="n">
+        <v>92.60316915016962</v>
+      </c>
+      <c r="K3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>0.8547185984544441</v>
-      </c>
-      <c r="G3" t="n">
+      <c r="M3" t="n">
+        <v>134</v>
+      </c>
+      <c r="N3" t="n">
+        <v>15</v>
+      </c>
+      <c r="O3" t="n">
         <v>163.2220354262268</v>
       </c>
-      <c r="H3" t="n">
+      <c r="P3" t="n">
         <v>10.88146902841512</v>
       </c>
-      <c r="I3" t="n">
-        <v>15</v>
-      </c>
-      <c r="J3" t="n">
-        <v>23287</v>
-      </c>
-      <c r="K3" t="n">
-        <v>1.356972204416992</v>
-      </c>
-      <c r="L3" t="n">
+      <c r="Q3" t="n">
         <v>3728</v>
       </c>
-      <c r="M3" t="n">
+      <c r="R3" t="n">
         <v>0.217236757764699</v>
       </c>
-      <c r="N3" t="n">
+      <c r="S3" t="n">
         <v>16.00893202215829</v>
       </c>
-      <c r="O3" t="n">
-        <v>6</v>
-      </c>
-      <c r="P3" t="n">
-        <v>134</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>2</v>
-      </c>
-      <c r="R3" t="n">
-        <v>67</v>
-      </c>
-      <c r="S3" t="n">
-        <v>92.60316915016962</v>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Ctrl</t>
+        </is>
+      </c>
+      <c r="U3" t="b">
+        <v>1</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="W3" t="n">
+        <v>106</v>
+      </c>
+      <c r="X3" t="n">
+        <v>29</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>196.5344549849193</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>6.777050171893769</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>5273</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>0.3072664763125692</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>22.6435350195388</v>
       </c>
     </row>
     <row r="4">
@@ -657,55 +775,89 @@
       <c r="C4" t="b">
         <v>1</v>
       </c>
-      <c r="D4" t="b">
-        <v>1</v>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="D4" t="n">
+        <v>0.8827156806926629</v>
+      </c>
+      <c r="E4" t="n">
+        <v>25388</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1.479400967309597</v>
+      </c>
+      <c r="G4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>42</v>
+      </c>
+      <c r="J4" t="n">
+        <v>76.44363478808886</v>
+      </c>
+      <c r="K4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="F4" t="n">
-        <v>0.8827156806926629</v>
-      </c>
-      <c r="G4" t="n">
+      <c r="M4" t="n">
+        <v>84</v>
+      </c>
+      <c r="N4" t="n">
+        <v>19</v>
+      </c>
+      <c r="O4" t="n">
         <v>139.5221817229474</v>
       </c>
-      <c r="H4" t="n">
+      <c r="P4" t="n">
         <v>7.34327272226039</v>
       </c>
-      <c r="I4" t="n">
-        <v>19</v>
-      </c>
-      <c r="J4" t="n">
-        <v>25388</v>
-      </c>
-      <c r="K4" t="n">
-        <v>1.479400967309597</v>
-      </c>
-      <c r="L4" t="n">
+      <c r="Q4" t="n">
         <v>7819</v>
       </c>
-      <c r="M4" t="n">
+      <c r="R4" t="n">
         <v>0.4556261290134608</v>
       </c>
-      <c r="N4" t="n">
+      <c r="S4" t="n">
         <v>30.79801481014652</v>
       </c>
-      <c r="O4" t="n">
-        <v>5</v>
-      </c>
-      <c r="P4" t="n">
-        <v>84</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R4" t="n">
-        <v>42</v>
-      </c>
-      <c r="S4" t="n">
-        <v>76.44363478808886</v>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Ctrl</t>
+        </is>
+      </c>
+      <c r="U4" t="b">
+        <v>1</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="W4" t="n">
+        <v>106</v>
+      </c>
+      <c r="X4" t="n">
+        <v>16</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>176.8967290960403</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>11.05604556850252</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>5231</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>0.3048190664879669</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>20.60422246730739</v>
       </c>
     </row>
     <row r="5">
@@ -722,55 +874,89 @@
       <c r="C5" t="b">
         <v>1</v>
       </c>
-      <c r="D5" t="b">
-        <v>1</v>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="D5" t="n">
+        <v>0.8657450241836028</v>
+      </c>
+      <c r="E5" t="n">
+        <v>25501</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1.485985665171027</v>
+      </c>
+      <c r="G5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>44</v>
+      </c>
+      <c r="J5" t="n">
+        <v>78.39810203521431</v>
+      </c>
+      <c r="K5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>0.8657450241836028</v>
-      </c>
-      <c r="G5" t="n">
+      <c r="M5" t="n">
+        <v>88</v>
+      </c>
+      <c r="N5" t="n">
+        <v>16</v>
+      </c>
+      <c r="O5" t="n">
         <v>126.431509133984</v>
       </c>
-      <c r="H5" t="n">
+      <c r="P5" t="n">
         <v>7.901969320873998</v>
       </c>
-      <c r="I5" t="n">
-        <v>16</v>
-      </c>
-      <c r="J5" t="n">
-        <v>25501</v>
-      </c>
-      <c r="K5" t="n">
-        <v>1.485985665171027</v>
-      </c>
-      <c r="L5" t="n">
+      <c r="Q5" t="n">
         <v>7904</v>
       </c>
-      <c r="M5" t="n">
+      <c r="R5" t="n">
         <v>0.4605792203251559</v>
       </c>
-      <c r="N5" t="n">
+      <c r="S5" t="n">
         <v>30.99486294655112</v>
       </c>
-      <c r="O5" t="n">
-        <v>6</v>
-      </c>
-      <c r="P5" t="n">
-        <v>88</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>1</v>
-      </c>
-      <c r="R5" t="n">
-        <v>44</v>
-      </c>
-      <c r="S5" t="n">
-        <v>78.39810203521431</v>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Ctrl</t>
+        </is>
+      </c>
+      <c r="U5" t="b">
+        <v>1</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="W5" t="n">
+        <v>106</v>
+      </c>
+      <c r="X5" t="n">
+        <v>15</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>132.9587087520175</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>8.863913916801165</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>6094</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>0.3551075112172951</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>23.89710207442845</v>
       </c>
     </row>
   </sheetData>

</xml_diff>